<commit_message>
finegray: refine estimator internals; expand QA suite
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_diagtab.xlsx
+++ b/tabtools/demo/demo_diagtab.xlsx
@@ -158,10 +158,10 @@
     <t>85.9%</t>
   </si>
   <si>
-    <t>(15.7, 16.4)</t>
-  </si>
-  <si>
-    <t>(85.7, 86.1)</t>
+    <t>(15.6, 16.5)</t>
+  </si>
+  <si>
+    <t>(85.5, 86.3)</t>
   </si>
   <si>
     <t>PPV and NPV adjusted to population prevalence of 15%.</t>

</xml_diff>

<commit_message>
qa: iivw add CR-ladder probes; tabtools release 1.12.0
To measure the unresolved FIPTIW interval scale and bound coverage claims
by tested scenarios, add `iivw_cr_ladder` in
`iivw/qa/_iivw_cr_ladder.do`, the `clubSandwich` cross-check in
`iivw/qa/crossval_cr_ladder.R`, and probe/test scripts wired through
`iivw/qa/run_all.do`; update the coverage plan and live SOL ledger while
leaving unrun P2-P5 and the FIPTIW interval method explicitly open.

Separately, bump tabtools to 1.12.0, synchronize version metadata in the
changed `.ado` and `.sthlp` files and both README files, revise
`_tabtools_csv_write.ado`, `comptab.ado`, `corrtab.ado`, and
`crosstab.ado`, and update the demo `.xlsx` artifacts.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_diagtab.xlsx
+++ b/tabtools/demo/demo_diagtab.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="709">
+  <fonts count="727">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1006,30 +1006,75 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
       <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1655,30 +1700,75 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
       <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
@@ -3262,7 +3352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="385">
+  <borders count="403">
     <border>
       <left/>
       <right/>
@@ -3851,22 +3941,85 @@
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -4443,22 +4596,85 @@
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -5890,7 +6106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="385">
+  <cellXfs count="403">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -6224,43 +6440,55 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="160" fillId="0" borderId="87" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="162" fillId="0" borderId="88" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="164" fillId="0" borderId="89" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="165" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="166" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="167" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0"/>
-    <xf numFmtId="0" fontId="169" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="171" fillId="0" borderId="98" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="173" fillId="0" borderId="99" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="159" fillId="0" borderId="87" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="160" fillId="0" borderId="88" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="161" fillId="0" borderId="89" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="162" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="163" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="164" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="166" fillId="0" borderId="93" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="168" fillId="0" borderId="94" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="170" fillId="0" borderId="95" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="171" fillId="0" borderId="96" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="172" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="173" fillId="0" borderId="98" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="174" fillId="0" borderId="99" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6268,1127 +6496,1187 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="177" fillId="0" borderId="101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="179" fillId="0" borderId="102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="181" fillId="0" borderId="103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="183" fillId="0" borderId="104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="185" fillId="0" borderId="105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="187" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="189" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="191" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="193" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="195" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="197" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="199" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="201" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="203" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="205" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="207" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="209" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="211" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="213" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="215" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="217" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="219" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="221" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="223" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="225" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="227" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="229" fillId="0" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="231" fillId="0" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="233" fillId="0" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="235" fillId="0" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="237" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="239" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="241" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="243" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="245" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="247" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="249" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="251" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="253" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="255" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="257" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="259" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="261" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="263" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="265" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="267" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="269" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="271" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="273" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="275" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="277" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="279" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="281" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="283" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="285" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="287" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="289" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="291" fillId="0" borderId="158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="293" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="295" fillId="0" borderId="160" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="297" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="299" fillId="0" borderId="162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="301" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="303" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="305" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="306" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="176" fillId="0" borderId="101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="102" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="103" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="104" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="105" xfId="0"/>
+    <xf numFmtId="0" fontId="178" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="180" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="182" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="184" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="186" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="188" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="190" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="192" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="194" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="196" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="198" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="200" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="202" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="204" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="206" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="208" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="210" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="212" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="214" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="216" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="218" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="220" fillId="0" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="222" fillId="0" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="224" fillId="0" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="226" fillId="0" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="228" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="230" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="232" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="234" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="236" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="238" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="240" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="242" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="244" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="246" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="248" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="250" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="252" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="254" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="256" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="258" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="260" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="262" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="264" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="266" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="268" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="270" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="272" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="274" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="276" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="278" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="280" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="282" fillId="0" borderId="158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="284" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="286" fillId="0" borderId="160" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="288" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="290" fillId="0" borderId="162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="292" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="294" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="296" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="298" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="300" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="302" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="304" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="306" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="308" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="310" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="312" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="314" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="315" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="307" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="316" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="308" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="317" fillId="0" borderId="177" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="310" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="312" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="314" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="315" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="319" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="321" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="323" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="324" fillId="0" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="316" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="325" fillId="0" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="317" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="326" fillId="0" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="319" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="321" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="323" fillId="0" borderId="177" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="324" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="325" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="326" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="327" fillId="0" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="327" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="328" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="329" fillId="0" borderId="186" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="330" fillId="0" borderId="187" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="331" fillId="0" borderId="188" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="332" fillId="0" borderId="189" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="334" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="336" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="338" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="339" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="340" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="341" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="342" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="343" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="344" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="345" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="328" fillId="0" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="346" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="329" fillId="0" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="347" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="331" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="349" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="333" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="351" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="186" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="187" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="188" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="189" xfId="0"/>
-    <xf numFmtId="0" fontId="335" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="337" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="339" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="341" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="343" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="345" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="347" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="349" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="351" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="353" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="355" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="357" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="359" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="361" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="363" fillId="0" borderId="204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="365" fillId="0" borderId="205" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="367" fillId="0" borderId="206" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="369" fillId="0" borderId="207" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="371" fillId="0" borderId="208" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="373" fillId="0" borderId="209" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="375" fillId="0" borderId="210" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="377" fillId="0" borderId="211" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="379" fillId="0" borderId="212" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="381" fillId="0" borderId="213" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="383" fillId="0" borderId="214" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="385" fillId="0" borderId="215" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="387" fillId="0" borderId="216" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="389" fillId="0" borderId="217" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="391" fillId="0" borderId="218" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="393" fillId="0" borderId="219" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="395" fillId="0" borderId="220" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="397" fillId="0" borderId="221" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="399" fillId="0" borderId="222" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="401" fillId="0" borderId="223" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="403" fillId="0" borderId="224" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="405" fillId="0" borderId="225" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="407" fillId="0" borderId="226" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="409" fillId="0" borderId="227" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="411" fillId="0" borderId="228" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="413" fillId="0" borderId="229" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="415" fillId="0" borderId="230" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="417" fillId="0" borderId="231" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="419" fillId="0" borderId="232" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="421" fillId="0" borderId="233" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="423" fillId="0" borderId="234" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="425" fillId="0" borderId="235" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="427" fillId="0" borderId="236" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="429" fillId="0" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="431" fillId="0" borderId="238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="433" fillId="0" borderId="239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="435" fillId="0" borderId="240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="437" fillId="0" borderId="241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="439" fillId="0" borderId="242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="441" fillId="0" borderId="243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="443" fillId="0" borderId="244" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="445" fillId="0" borderId="245" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="447" fillId="0" borderId="246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="449" fillId="0" borderId="247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="451" fillId="0" borderId="248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="453" fillId="0" borderId="249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="455" fillId="0" borderId="250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="457" fillId="0" borderId="251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="459" fillId="0" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="461" fillId="0" borderId="253" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="463" fillId="0" borderId="254" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="465" fillId="0" borderId="255" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="467" fillId="0" borderId="256" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="469" fillId="0" borderId="257" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="471" fillId="0" borderId="258" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="473" fillId="0" borderId="259" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="475" fillId="0" borderId="260" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="477" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="479" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="481" fillId="0" borderId="263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="483" fillId="0" borderId="264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="485" fillId="0" borderId="265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="487" fillId="0" borderId="266" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="489" fillId="0" borderId="267" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="491" fillId="0" borderId="268" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="493" fillId="0" borderId="269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="495" fillId="0" borderId="270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="497" fillId="0" borderId="271" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="499" fillId="0" borderId="272" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="501" fillId="0" borderId="273" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="503" fillId="0" borderId="274" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="505" fillId="0" borderId="275" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="507" fillId="0" borderId="276" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="509" fillId="0" borderId="277" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="511" fillId="0" borderId="278" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="513" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="515" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="517" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="519" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="521" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="523" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="525" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="527" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="529" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="531" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="533" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="535" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="537" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="539" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="541" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="543" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="545" fillId="0" borderId="295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="547" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="549" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="551" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="553" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="555" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="557" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="559" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="561" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="563" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="565" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="567" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="569" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="571" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="573" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="575" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="577" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="579" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="581" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="583" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="585" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="587" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="589" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="591" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="593" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="595" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="597" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="599" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="601" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="603" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="605" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="607" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="609" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="611" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="613" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="615" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="617" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="619" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="621" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="623" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="625" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="627" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="629" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="631" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="633" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="635" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="637" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="639" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="641" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="643" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="645" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="647" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="648" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="204" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="205" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="206" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="207" xfId="0"/>
+    <xf numFmtId="0" fontId="353" fillId="0" borderId="208" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="355" fillId="0" borderId="209" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="357" fillId="0" borderId="210" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="359" fillId="0" borderId="211" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="361" fillId="0" borderId="212" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="363" fillId="0" borderId="213" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="365" fillId="0" borderId="214" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="367" fillId="0" borderId="215" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="369" fillId="0" borderId="216" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="371" fillId="0" borderId="217" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="373" fillId="0" borderId="218" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="375" fillId="0" borderId="219" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="377" fillId="0" borderId="220" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="379" fillId="0" borderId="221" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="381" fillId="0" borderId="222" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="383" fillId="0" borderId="223" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="385" fillId="0" borderId="224" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="387" fillId="0" borderId="225" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="389" fillId="0" borderId="226" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="391" fillId="0" borderId="227" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="393" fillId="0" borderId="228" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="395" fillId="0" borderId="229" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="397" fillId="0" borderId="230" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="399" fillId="0" borderId="231" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="401" fillId="0" borderId="232" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="403" fillId="0" borderId="233" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="405" fillId="0" borderId="234" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="407" fillId="0" borderId="235" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="409" fillId="0" borderId="236" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="411" fillId="0" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="413" fillId="0" borderId="238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="415" fillId="0" borderId="239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="417" fillId="0" borderId="240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="419" fillId="0" borderId="241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="421" fillId="0" borderId="242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="423" fillId="0" borderId="243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="425" fillId="0" borderId="244" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="427" fillId="0" borderId="245" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="429" fillId="0" borderId="246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="431" fillId="0" borderId="247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="433" fillId="0" borderId="248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="435" fillId="0" borderId="249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="437" fillId="0" borderId="250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="439" fillId="0" borderId="251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="441" fillId="0" borderId="252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="443" fillId="0" borderId="253" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="445" fillId="0" borderId="254" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="447" fillId="0" borderId="255" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="449" fillId="0" borderId="256" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="451" fillId="0" borderId="257" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="453" fillId="0" borderId="258" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="455" fillId="0" borderId="259" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="457" fillId="0" borderId="260" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="459" fillId="0" borderId="261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="461" fillId="0" borderId="262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="463" fillId="0" borderId="263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="465" fillId="0" borderId="264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="467" fillId="0" borderId="265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="469" fillId="0" borderId="266" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="471" fillId="0" borderId="267" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="473" fillId="0" borderId="268" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="475" fillId="0" borderId="269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="477" fillId="0" borderId="270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="479" fillId="0" borderId="271" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="481" fillId="0" borderId="272" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="483" fillId="0" borderId="273" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="485" fillId="0" borderId="274" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="487" fillId="0" borderId="275" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="489" fillId="0" borderId="276" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="491" fillId="0" borderId="277" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="493" fillId="0" borderId="278" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="495" fillId="0" borderId="279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="497" fillId="0" borderId="280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="499" fillId="0" borderId="281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="501" fillId="0" borderId="282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="503" fillId="0" borderId="283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="505" fillId="0" borderId="284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="507" fillId="0" borderId="285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="509" fillId="0" borderId="286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="511" fillId="0" borderId="287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="513" fillId="0" borderId="288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="515" fillId="0" borderId="289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="517" fillId="0" borderId="290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="519" fillId="0" borderId="291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="521" fillId="0" borderId="292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="523" fillId="0" borderId="293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="525" fillId="0" borderId="294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="527" fillId="0" borderId="295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="529" fillId="0" borderId="296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="531" fillId="0" borderId="297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="533" fillId="0" borderId="298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="535" fillId="0" borderId="299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="537" fillId="0" borderId="300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="539" fillId="0" borderId="301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="541" fillId="0" borderId="302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="543" fillId="0" borderId="303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="545" fillId="0" borderId="304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="547" fillId="0" borderId="305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="549" fillId="0" borderId="306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="551" fillId="0" borderId="307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="553" fillId="0" borderId="308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="555" fillId="0" borderId="309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="557" fillId="0" borderId="310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="559" fillId="0" borderId="311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="561" fillId="0" borderId="312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="563" fillId="0" borderId="313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="565" fillId="0" borderId="314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="567" fillId="0" borderId="315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="569" fillId="0" borderId="316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="571" fillId="0" borderId="317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="573" fillId="0" borderId="318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="575" fillId="0" borderId="319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="577" fillId="0" borderId="320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="579" fillId="0" borderId="321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="581" fillId="0" borderId="322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="583" fillId="0" borderId="323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="585" fillId="0" borderId="324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="587" fillId="0" borderId="325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="589" fillId="0" borderId="326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="591" fillId="0" borderId="327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="593" fillId="0" borderId="328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="595" fillId="0" borderId="329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="597" fillId="0" borderId="330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="599" fillId="0" borderId="331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="601" fillId="0" borderId="332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="603" fillId="0" borderId="333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="605" fillId="0" borderId="334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="607" fillId="0" borderId="335" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="609" fillId="0" borderId="336" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="611" fillId="0" borderId="337" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="613" fillId="0" borderId="338" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="615" fillId="0" borderId="339" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="617" fillId="0" borderId="340" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="619" fillId="0" borderId="341" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="621" fillId="0" borderId="342" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="623" fillId="0" borderId="343" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="625" fillId="0" borderId="344" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="627" fillId="0" borderId="345" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="629" fillId="0" borderId="346" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="631" fillId="0" borderId="347" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="633" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="635" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="637" fillId="0" borderId="350" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="639" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="641" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="643" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="645" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="647" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="649" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="651" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="653" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="655" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="657" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="659" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="661" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="663" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="665" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="666" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="649" fillId="0" borderId="348" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="667" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="650" fillId="0" borderId="349" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="668" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="652" fillId="0" borderId="350" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="654" fillId="0" borderId="351" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="656" fillId="0" borderId="352" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="657" fillId="0" borderId="353" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="670" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="672" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="674" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="675" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="658" fillId="0" borderId="354" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="676" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="659" fillId="0" borderId="355" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="677" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="660" fillId="0" borderId="356" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="678" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="661" fillId="0" borderId="357" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="679" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="662" fillId="0" borderId="358" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="680" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="664" fillId="0" borderId="359" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="666" fillId="0" borderId="360" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="668" fillId="0" borderId="361" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="670" fillId="0" borderId="362" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="672" fillId="0" borderId="363" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="674" fillId="0" borderId="364" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="676" fillId="0" borderId="365" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="678" fillId="0" borderId="366" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="680" fillId="0" borderId="367" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="682" fillId="0" borderId="368" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="684" fillId="0" borderId="369" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="686" fillId="0" borderId="370" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="688" fillId="0" borderId="371" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="690" fillId="0" borderId="372" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="692" fillId="0" borderId="373" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="694" fillId="0" borderId="374" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="696" fillId="0" borderId="375" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="698" fillId="0" borderId="376" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="699" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="700" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="701" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="702" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="682" fillId="0" borderId="377" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="684" fillId="0" borderId="378" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="686" fillId="0" borderId="379" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="688" fillId="0" borderId="380" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="690" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="692" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="694" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="696" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="698" fillId="0" borderId="385" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="700" fillId="0" borderId="386" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="702" fillId="0" borderId="387" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="704" fillId="0" borderId="388" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="706" fillId="0" borderId="389" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="708" fillId="0" borderId="390" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="710" fillId="0" borderId="391" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="712" fillId="0" borderId="392" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="714" fillId="0" borderId="393" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="716" fillId="0" borderId="394" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="717" fillId="0" borderId="395" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="718" fillId="0" borderId="396" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="719" fillId="0" borderId="397" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="720" fillId="0" borderId="398" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="703" fillId="0" borderId="381" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="721" fillId="0" borderId="399" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="704" fillId="0" borderId="382" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="722" fillId="0" borderId="400" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="706" fillId="0" borderId="383" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="724" fillId="0" borderId="401" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="708" fillId="0" borderId="384" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="726" fillId="0" borderId="402" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7428,13 +7716,13 @@
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="84" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="85" t="s">
+      <c r="B2" s="90" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="86" t="s">
+      <c r="D2" s="92" t="s">
         <v>31</v>
       </c>
     </row>
@@ -7484,13 +7772,13 @@
       <c r="A6" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="87" t="s">
+      <c r="B6" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="88" t="s">
+      <c r="C6" s="97" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="89" t="s">
+      <c r="D6" s="98" t="s">
         <v>34</v>
       </c>
     </row>
@@ -7638,13 +7926,13 @@
       <c r="A17" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="90" t="s">
+      <c r="B17" s="99" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="91" t="s">
+      <c r="C17" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="92" t="s">
+      <c r="D17" s="101" t="s">
         <v>1</v>
       </c>
     </row>
@@ -7660,238 +7948,238 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="93" customWidth="true"/>
-    <col min="2" max="2" width="18.7109375" style="94" customWidth="true"/>
-    <col min="3" max="3" width="12.7109375" style="95" customWidth="true"/>
-    <col min="4" max="4" width="18.7109375" style="96" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="102" customWidth="true"/>
+    <col min="2" max="2" width="18.7109375" style="103" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" style="104" customWidth="true"/>
+    <col min="4" max="4" width="18.7109375" style="105" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="168" t="s">
+      <c r="A1" s="177" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="161" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="161" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="161" t="s">
+      <c r="B1" s="170" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="170" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="170" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="101" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="172" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="173" t="s">
+      <c r="A2" s="110" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="187" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="188" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="174" t="s">
+      <c r="D2" s="189" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="105" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="106" t="s">
+      <c r="A3" s="114" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="107" t="s">
+      <c r="C3" s="116" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="108" t="s">
+      <c r="D3" s="117" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="109" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="110" t="s">
+      <c r="A4" s="118" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="119" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="111" t="s">
+      <c r="C4" s="120" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="112" t="s">
+      <c r="D4" s="121" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="113" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="114" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="115" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="116" t="s">
+      <c r="A5" s="122" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="123" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="124" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="125" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="117" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="175" t="s">
+      <c r="A6" s="126" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="193" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="176" t="s">
+      <c r="C6" s="194" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="177" t="s">
+      <c r="D6" s="195" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="121" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="122" t="s">
+      <c r="A7" s="130" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="131" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="123" t="s">
+      <c r="C7" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="124" t="s">
+      <c r="D7" s="133" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="125" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="126" t="s">
+      <c r="A8" s="134" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="135" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="127" t="s">
+      <c r="C8" s="136" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="128" t="s">
+      <c r="D8" s="137" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="129" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="130" t="s">
+      <c r="A9" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="139" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="131" t="s">
+      <c r="C9" s="140" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="132" t="s">
+      <c r="D9" s="141" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="133" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="134" t="s">
+      <c r="A10" s="142" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="143" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="135" t="s">
+      <c r="C10" s="144" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="136" t="s">
+      <c r="D10" s="145" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="137" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="138" t="s">
+      <c r="A11" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="147" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="139" t="s">
+      <c r="C11" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="140" t="s">
+      <c r="D11" s="149" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="141" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="142" t="s">
+      <c r="A12" s="150" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="151" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="143" t="s">
+      <c r="C12" s="152" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="144" t="s">
+      <c r="D12" s="153" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="145" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="146" t="s">
+      <c r="A13" s="154" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="155" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="147" t="s">
+      <c r="C13" s="156" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="148" t="s">
+      <c r="D13" s="157" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="149" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="150" t="s">
+      <c r="A14" s="158" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="159" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="151" t="s">
+      <c r="C14" s="160" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="152" t="s">
+      <c r="D14" s="161" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="153" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="154" t="s">
+      <c r="A15" s="162" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="163" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="155" t="s">
+      <c r="C15" s="164" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="156" t="s">
+      <c r="D15" s="165" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="157" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="178" t="s">
+      <c r="A16" s="166" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="196" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="179" t="s">
+      <c r="C16" s="197" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="180" t="s">
+      <c r="D16" s="198" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="185" t="s">
+      <c r="B17" s="203" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="0"/>
@@ -7910,546 +8198,546 @@
   <dimension ref="A1:D39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="186" customWidth="true"/>
-    <col min="2" max="2" width="18.7109375" style="187" customWidth="true"/>
-    <col min="3" max="3" width="12.7109375" style="188" customWidth="true"/>
-    <col min="4" max="4" width="18.7109375" style="189" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="204" customWidth="true"/>
+    <col min="2" max="2" width="18.7109375" style="205" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" style="206" customWidth="true"/>
+    <col min="4" max="4" width="18.7109375" style="207" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="349" t="s">
+      <c r="A1" s="367" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="342" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="342" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="342" t="s">
+      <c r="B1" s="360" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="360" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="360" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="194" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="356" t="s">
+      <c r="A2" s="212" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="374" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="357" t="s">
+      <c r="C2" s="375" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="358" t="s">
+      <c r="D2" s="376" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="198" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="359" t="s">
+      <c r="A3" s="216" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="377" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="360" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="361" t="s">
+      <c r="C3" s="378" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="379" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="202" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="203" t="s">
+      <c r="A4" s="220" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="221" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="204" t="s">
+      <c r="C4" s="222" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="205" t="s">
+      <c r="D4" s="223" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="206" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="207" t="s">
+      <c r="A5" s="224" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="225" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="208" t="s">
+      <c r="C5" s="226" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="209" t="s">
+      <c r="D5" s="227" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="210" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="211" t="s">
+      <c r="A6" s="228" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="229" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="212" t="s">
+      <c r="C6" s="230" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="213" t="s">
+      <c r="D6" s="231" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="214" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="215" t="s">
+      <c r="A7" s="232" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="233" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="216" t="s">
+      <c r="C7" s="234" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="217" t="s">
+      <c r="D7" s="235" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="218" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="219" t="s">
+      <c r="A8" s="236" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="237" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="220" t="s">
+      <c r="C8" s="238" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="221" t="s">
+      <c r="D8" s="239" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="222" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="362" t="s">
+      <c r="A9" s="240" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="380" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="363" t="s">
-        <v>1</v>
-      </c>
-      <c r="D9" s="364" t="s">
+      <c r="C9" s="381" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="382" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="226" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="227" t="s">
+      <c r="A10" s="244" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="245" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="228" t="s">
+      <c r="C10" s="246" t="s">
         <v>67</v>
       </c>
-      <c r="D10" s="229" t="s">
+      <c r="D10" s="247" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="230" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="231" t="s">
+      <c r="A11" s="248" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="249" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="232" t="s">
+      <c r="C11" s="250" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="233" t="s">
+      <c r="D11" s="251" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="234" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="235" t="s">
+      <c r="A12" s="252" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="253" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="236" t="s">
+      <c r="C12" s="254" t="s">
         <v>69</v>
       </c>
-      <c r="D12" s="237" t="s">
+      <c r="D12" s="255" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="238" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="239" t="s">
+      <c r="A13" s="256" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="257" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="240" t="s">
+      <c r="C13" s="258" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="241" t="s">
+      <c r="D13" s="259" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="242" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="243" t="s">
+      <c r="A14" s="260" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="261" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="244" t="s">
+      <c r="C14" s="262" t="s">
         <v>71</v>
       </c>
-      <c r="D14" s="245" t="s">
+      <c r="D14" s="263" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="246" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="365" t="s">
+      <c r="A15" s="264" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="383" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="366" t="s">
-        <v>1</v>
-      </c>
-      <c r="D15" s="367" t="s">
+      <c r="C15" s="384" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="385" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="250" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="251" t="s">
+      <c r="A16" s="268" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="269" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="252" t="s">
+      <c r="C16" s="270" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="253" t="s">
+      <c r="D16" s="271" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="254" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="255" t="s">
+      <c r="A17" s="272" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="273" t="s">
         <v>54</v>
       </c>
-      <c r="C17" s="256" t="s">
+      <c r="C17" s="274" t="s">
         <v>73</v>
       </c>
-      <c r="D17" s="257" t="s">
+      <c r="D17" s="275" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="258" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="259" t="s">
+      <c r="A18" s="276" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="277" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="260" t="s">
+      <c r="C18" s="278" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="261" t="s">
+      <c r="D18" s="279" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="262" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="263" t="s">
+      <c r="A19" s="280" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="281" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="264" t="s">
+      <c r="C19" s="282" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="265" t="s">
+      <c r="D19" s="283" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="266" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="267" t="s">
+      <c r="A20" s="284" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="285" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="268" t="s">
+      <c r="C20" s="286" t="s">
         <v>75</v>
       </c>
-      <c r="D20" s="269" t="s">
+      <c r="D20" s="287" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="270" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="368" t="s">
+      <c r="A21" s="288" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="386" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="369" t="s">
-        <v>1</v>
-      </c>
-      <c r="D21" s="370" t="s">
+      <c r="C21" s="387" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="388" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="274" t="s">
-        <v>1</v>
-      </c>
-      <c r="B22" s="275" t="s">
+      <c r="A22" s="292" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="293" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="276" t="s">
+      <c r="C22" s="294" t="s">
         <v>76</v>
       </c>
-      <c r="D22" s="277" t="s">
+      <c r="D22" s="295" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="278" t="s">
-        <v>1</v>
-      </c>
-      <c r="B23" s="279" t="s">
+      <c r="A23" s="296" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="297" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="280" t="s">
+      <c r="C23" s="298" t="s">
         <v>77</v>
       </c>
-      <c r="D23" s="281" t="s">
+      <c r="D23" s="299" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="282" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="283" t="s">
+      <c r="A24" s="300" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="301" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="284" t="s">
+      <c r="C24" s="302" t="s">
         <v>78</v>
       </c>
-      <c r="D24" s="285" t="s">
+      <c r="D24" s="303" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="286" t="s">
-        <v>1</v>
-      </c>
-      <c r="B25" s="287" t="s">
+      <c r="A25" s="304" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="305" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="288" t="s">
+      <c r="C25" s="306" t="s">
         <v>79</v>
       </c>
-      <c r="D25" s="289" t="s">
+      <c r="D25" s="307" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="290" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="291" t="s">
+      <c r="A26" s="308" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="309" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="292" t="s">
+      <c r="C26" s="310" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="293" t="s">
+      <c r="D26" s="311" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="294" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="371" t="s">
+      <c r="A27" s="312" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="389" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="372" t="s">
-        <v>1</v>
-      </c>
-      <c r="D27" s="373" t="s">
+      <c r="C27" s="390" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="391" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="298" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="299" t="s">
+      <c r="A28" s="316" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="317" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="300" t="s">
+      <c r="C28" s="318" t="s">
         <v>81</v>
       </c>
-      <c r="D28" s="301" t="s">
+      <c r="D28" s="319" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="302" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="303" t="s">
+      <c r="A29" s="320" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="321" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="304" t="s">
+      <c r="C29" s="322" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="305" t="s">
+      <c r="D29" s="323" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="306" t="s">
-        <v>1</v>
-      </c>
-      <c r="B30" s="307" t="s">
+      <c r="A30" s="324" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="325" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="308" t="s">
+      <c r="C30" s="326" t="s">
         <v>83</v>
       </c>
-      <c r="D30" s="309" t="s">
+      <c r="D30" s="327" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="310" t="s">
-        <v>1</v>
-      </c>
-      <c r="B31" s="311" t="s">
+      <c r="A31" s="328" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="329" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="312" t="s">
+      <c r="C31" s="330" t="s">
         <v>84</v>
       </c>
-      <c r="D31" s="313" t="s">
+      <c r="D31" s="331" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="314" t="s">
-        <v>1</v>
-      </c>
-      <c r="B32" s="315" t="s">
+      <c r="A32" s="332" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="333" t="s">
         <v>57</v>
       </c>
-      <c r="C32" s="316" t="s">
+      <c r="C32" s="334" t="s">
         <v>85</v>
       </c>
-      <c r="D32" s="317" t="s">
+      <c r="D32" s="335" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="318" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="374" t="s">
+      <c r="A33" s="336" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="392" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="375" t="s">
-        <v>1</v>
-      </c>
-      <c r="D33" s="376" t="s">
+      <c r="C33" s="393" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="394" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="322" t="s">
-        <v>1</v>
-      </c>
-      <c r="B34" s="323" t="s">
+      <c r="A34" s="340" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="341" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="324" t="s">
+      <c r="C34" s="342" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="325" t="s">
+      <c r="D34" s="343" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="326" t="s">
-        <v>1</v>
-      </c>
-      <c r="B35" s="327" t="s">
+      <c r="A35" s="344" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="345" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="328" t="s">
+      <c r="C35" s="346" t="s">
         <v>63</v>
       </c>
-      <c r="D35" s="329" t="s">
+      <c r="D35" s="347" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="330" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="331" t="s">
+      <c r="A36" s="348" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="349" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="332" t="s">
+      <c r="C36" s="350" t="s">
         <v>66</v>
       </c>
-      <c r="D36" s="333" t="s">
+      <c r="D36" s="351" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="334" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="335" t="s">
+      <c r="A37" s="352" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="353" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="336" t="s">
+      <c r="C37" s="354" t="s">
         <v>84</v>
       </c>
-      <c r="D37" s="337" t="s">
+      <c r="D37" s="355" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="338" t="s">
-        <v>1</v>
-      </c>
-      <c r="B38" s="377" t="s">
+      <c r="A38" s="356" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="395" t="s">
         <v>57</v>
       </c>
-      <c r="C38" s="378" t="s">
+      <c r="C38" s="396" t="s">
         <v>84</v>
       </c>
-      <c r="D38" s="379" t="s">
+      <c r="D38" s="397" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="384" t="s">
+      <c r="B39" s="402" t="s">
         <v>111</v>
       </c>
       <c r="C39" s="0"/>

</xml_diff>